<commit_message>
update rekap nilai dan konten blog
</commit_message>
<xml_diff>
--- a/Nilai PTS dan ASAS Ganjil 2025-2026/Olah Nilai ASAS/XI ASAS/SOAL PAS INFORMATIKA SMT GANJIL TH.2025_2026  (Jawaban).xlsx
+++ b/Nilai PTS dan ASAS Ganjil 2025-2026/Olah Nilai ASAS/XI ASAS/SOAL PAS INFORMATIKA SMT GANJIL TH.2025_2026  (Jawaban).xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="12840" windowHeight="11950" activeTab="1"/>
+    <workbookView windowWidth="27150" windowHeight="11950" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="XI-3" sheetId="2" r:id="rId1"/>
@@ -666,7 +666,7 @@
     <numFmt numFmtId="178" formatCode="m/d/yyyy\ h:mm:ss"/>
     <numFmt numFmtId="179" formatCode="0.00_);[Red]\(0.00\)"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="23">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -680,6 +680,12 @@
       <name val="Arial"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1136,31 +1142,28 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1169,119 +1172,122 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1301,6 +1307,7 @@
     <xf numFmtId="179" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" quotePrefix="1">
       <alignment vertical="center"/>
     </xf>
@@ -1363,7 +1370,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1377,7 +1384,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1391,7 +1398,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1405,7 +1412,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1419,7 +1426,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1433,7 +1440,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1447,7 +1454,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1461,7 +1468,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1475,7 +1482,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1489,7 +1496,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1503,7 +1510,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1517,7 +1524,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1531,7 +1538,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1545,7 +1552,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1559,7 +1566,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1573,7 +1580,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1587,7 +1594,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1601,7 +1608,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1615,7 +1622,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1629,7 +1636,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1643,7 +1650,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1657,7 +1664,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1671,7 +1678,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1685,7 +1692,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1699,7 +1706,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1713,7 +1720,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1727,7 +1734,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1741,7 +1748,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1755,7 +1762,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1769,7 +1776,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1783,7 +1790,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1797,7 +1804,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1811,7 +1818,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1825,7 +1832,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1839,7 +1846,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1853,7 +1860,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1867,7 +1874,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1881,7 +1888,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1895,7 +1902,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1909,7 +1916,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1923,7 +1930,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1937,7 +1944,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1952,7 +1959,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1967,7 +1974,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1981,7 +1988,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -1995,7 +2002,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2009,7 +2016,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2023,7 +2030,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2037,7 +2044,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2051,7 +2058,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2065,7 +2072,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2079,7 +2086,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2093,7 +2100,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2107,7 +2114,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2121,7 +2128,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2135,7 +2142,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2149,7 +2156,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2163,7 +2170,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2177,7 +2184,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2191,7 +2198,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2205,7 +2212,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2219,7 +2226,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2233,7 +2240,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2247,7 +2254,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2261,7 +2268,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2275,7 +2282,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2289,7 +2296,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2303,7 +2310,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2317,7 +2324,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2331,7 +2338,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2345,7 +2352,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2359,7 +2366,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2373,7 +2380,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2387,7 +2394,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2401,7 +2408,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2415,7 +2422,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2429,7 +2436,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2443,7 +2450,7 @@
     <dxf>
       <font>
         <name val="Arial"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
         <charset val="134"/>
         <family val="0"/>
         <b val="0"/>
@@ -2496,7 +2503,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1">
-    <tableStyle name="Form Responses 1-style" pivot="0" count="4" xr9:uid="{CBF71D18-07FA-DC77-288D-2E694826DD6C}">
+    <tableStyle name="Form Responses 1-style" pivot="0" count="4" xr9:uid="{8E6073C6-9B71-72CF-9D8E-326924F71636}">
       <tableStyleElement type="wholeTable" dxfId="81"/>
       <tableStyleElement type="headerRow" dxfId="80"/>
       <tableStyleElement type="firstRowStripe" dxfId="79"/>
@@ -2882,6 +2889,11 @@
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="zero"/>
     <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext uri="{0b15fc19-7d7d-44ad-8c2d-2c3a37ce22c3}">
+        <chartProps xmlns="https://web.wps.cn/et/2018/main" chartId="{442c1c47-86d3-4c6d-a9e1-92b65265cb11}"/>
+      </c:ext>
+    </c:extLst>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -3274,6 +3286,11 @@
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext uri="{0b15fc19-7d7d-44ad-8c2d-2c3a37ce22c3}">
+        <chartProps xmlns="https://web.wps.cn/et/2018/main" chartId="{77f9d29c-061a-475e-9a59-7207d5eb8661}"/>
+      </c:ext>
+    </c:extLst>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -4470,8 +4487,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Form_Responses3" displayName="Form_Responses3" ref="A1:AM40">
-  <sortState ref="A2:AM40">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Form_Responses3" displayName="Form_Responses3" ref="A1:AM41">
+  <sortState ref="A1:AM41">
     <sortCondition ref="E2:E40"/>
   </sortState>
   <tableColumns count="39">
@@ -4521,7 +4538,7 @@
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Form_Responses" displayName="Form_Responses" ref="A1:AM36">
-  <sortState ref="A2:AM36">
+  <sortState ref="A1:AM36">
     <sortCondition ref="E2:E36"/>
   </sortState>
   <tableColumns count="39">
@@ -5054,7 +5071,7 @@
       <c r="C3" s="6">
         <v>91</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="8" t="s">
         <v>75</v>
       </c>
       <c r="E3" s="5" t="s">
@@ -5173,7 +5190,7 @@
       <c r="C4" s="6">
         <v>94</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="8" t="s">
         <v>78</v>
       </c>
       <c r="E4" s="5" t="s">
@@ -5530,7 +5547,7 @@
       <c r="C7" s="6">
         <v>88</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="8" t="s">
         <v>82</v>
       </c>
       <c r="E7" s="5" t="s">
@@ -5887,7 +5904,7 @@
       <c r="C10" s="6">
         <v>79</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="8" t="s">
         <v>92</v>
       </c>
       <c r="E10" s="5" t="s">
@@ -9566,7 +9583,47 @@
         <v>74</v>
       </c>
     </row>
-    <row r="41" ht="22.5" customHeight="1"/>
+    <row r="41" ht="22.5" customHeight="1" spans="1:39">
+      <c r="A41" s="7"/>
+      <c r="B41" s="7"/>
+      <c r="C41" s="7"/>
+      <c r="D41" s="7"/>
+      <c r="E41" s="7"/>
+      <c r="F41" s="7"/>
+      <c r="G41" s="7"/>
+      <c r="H41" s="7"/>
+      <c r="I41" s="7"/>
+      <c r="J41" s="7"/>
+      <c r="K41" s="7"/>
+      <c r="L41" s="7"/>
+      <c r="M41" s="7"/>
+      <c r="N41" s="7"/>
+      <c r="O41" s="7"/>
+      <c r="P41" s="7"/>
+      <c r="Q41" s="7"/>
+      <c r="R41" s="7"/>
+      <c r="S41" s="7"/>
+      <c r="T41" s="7"/>
+      <c r="U41" s="7"/>
+      <c r="V41" s="7"/>
+      <c r="W41" s="7"/>
+      <c r="X41" s="7"/>
+      <c r="Y41" s="7"/>
+      <c r="Z41" s="7"/>
+      <c r="AA41" s="7"/>
+      <c r="AB41" s="7"/>
+      <c r="AC41" s="7"/>
+      <c r="AD41" s="7"/>
+      <c r="AE41" s="7"/>
+      <c r="AF41" s="7"/>
+      <c r="AG41" s="7"/>
+      <c r="AH41" s="7"/>
+      <c r="AI41" s="7"/>
+      <c r="AJ41" s="7"/>
+      <c r="AK41" s="7"/>
+      <c r="AL41" s="7"/>
+      <c r="AM41" s="7"/>
+    </row>
     <row r="42" ht="22.5" customHeight="1"/>
     <row r="43" ht="22.5" customHeight="1"/>
     <row r="44" ht="22.5" customHeight="1"/>
@@ -9848,7 +9905,7 @@
       <c r="C2" s="6">
         <v>88</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="9" t="s">
         <v>152</v>
       </c>
       <c r="E2" s="5" t="s">
@@ -9967,7 +10024,7 @@
       <c r="C3" s="6">
         <v>94</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="9" t="s">
         <v>75</v>
       </c>
       <c r="E3" s="5" t="s">
@@ -10324,7 +10381,7 @@
       <c r="C6" s="6">
         <v>94</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="9" t="s">
         <v>164</v>
       </c>
       <c r="E6" s="5" t="s">
@@ -10800,7 +10857,7 @@
       <c r="C10" s="6">
         <v>91</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="9" t="s">
         <v>92</v>
       </c>
       <c r="E10" s="5" t="s">

</xml_diff>